<commit_message>
Rebuild every figure on a shared journal style, one script per figure
</commit_message>
<xml_diff>
--- a/figures/excel/Table_S1.xlsx
+++ b/figures/excel/Table_S1.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,11 +32,6 @@
       <sz val="10"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
       <sz val="10"/>
     </font>
     <font>
@@ -44,20 +39,15 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -67,16 +57,30 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00000000"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00000000"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00000000"/>
       </bottom>
     </border>
   </borders>
@@ -88,13 +92,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>

</xml_diff>